<commit_message>
Fix dictionary gml:id to match schema code-carrying elements
The Dictionary gml:id must be the DIGGS element that carries the code
(as get_defined_codeTypes.js derives the validation XPath from it), not
the file name.

- cpt_interpreted_properties: gml:id propertyClass (interpreted CPT values
  are propertyClass codes on the measurement Property, like the raw
  channels), confirmed against Diggs.xsd PropertyType.
- cpt_interpretation_methods: gml:id correctionUsed and scoped to
  StaticConePenetrationTest. DIGGS 2.6 has no dedicated interpretation-
  method element; Property/correctionUsed is the CodeType hook for an
  adjustment/derivation used to obtain a reported result.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Codelist Excel Files and Conversion Templates to XML/cpt_interpretation_methods.xlsx
+++ b/Codelist Excel Files and Conversion Templates to XML/cpt_interpretation_methods.xlsx
@@ -966,7 +966,7 @@
     <row r="3" ht="154" customFormat="1" customHeight="1" s="2">
       <c r="B3" t="inlineStr">
         <is>
-          <t>cpt_interpretation_methods</t>
+          <t>correctionUsed</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -1271,7 +1271,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D1"/>
+  <dimension ref="A1:D10"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="10.83203125" defaultRowHeight="16"/>
   <cols>
     <col width="6.83203125" customWidth="1" min="1" max="1"/>
@@ -1299,6 +1299,159 @@
       <c r="D1" s="6" t="inlineStr">
         <is>
           <t>ConditionalElement</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>robertson_1986</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>//diggs:correctionUsed</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>ancestor::diggs:measurement//diggs:procedure/diggs:StaticConePenetrationTest</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>robertson_wride_1998</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>//diggs:correctionUsed</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>ancestor::diggs:measurement//diggs:procedure/diggs:StaticConePenetrationTest</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>robertson_1990</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>//diggs:correctionUsed</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>ancestor::diggs:measurement//diggs:procedure/diggs:StaticConePenetrationTest</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>robertson_2009</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>//diggs:correctionUsed</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>ancestor::diggs:measurement//diggs:procedure/diggs:StaticConePenetrationTest</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>robertson_2010</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>//diggs:correctionUsed</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>ancestor::diggs:measurement//diggs:procedure/diggs:StaticConePenetrationTest</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>jamiolkowski_2003</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>//diggs:correctionUsed</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>ancestor::diggs:measurement//diggs:procedure/diggs:StaticConePenetrationTest</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>kulhawy_mayne_1990</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>//diggs:correctionUsed</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>ancestor::diggs:measurement//diggs:procedure/diggs:StaticConePenetrationTest</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>su_nkt</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>//diggs:correctionUsed</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>ancestor::diggs:measurement//diggs:procedure/diggs:StaticConePenetrationTest</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>unit_weight_sbt_zone</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>//diggs:correctionUsed</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>ancestor::diggs:measurement//diggs:procedure/diggs:StaticConePenetrationTest</t>
         </is>
       </c>
     </row>

</xml_diff>